<commit_message>
feat!: write datetime.time as a fraction of a day
Excel's own time representation, so =A2*24 now works. Time cells in the
dtype templates carry an hh:mm:ss format so read-back stays exact. Golden
files regenerated (no time cells changed; stale autoFilter refs refreshed).
</commit_message>
<xml_diff>
--- a/tests/assets/golden/openpyxl/test_template_2_charts_filled.xlsx
+++ b/tests/assets/golden/openpyxl/test_template_2_charts_filled.xlsx
@@ -4432,7 +4432,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ColumnChartTable" displayName="ColumnChartTable" ref="A1:E4" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:E5"/>
+  <autoFilter ref="A1:E4"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Region"/>
     <tableColumn id="2" name="Q1"/>
@@ -4446,7 +4446,7 @@
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="WaterfallChartTable" displayName="WaterfallChartTable" ref="A1:B5" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:B9"/>
+  <autoFilter ref="A1:B5"/>
   <tableColumns count="2">
     <tableColumn id="1" name="Category"/>
     <tableColumn id="2" name="Amount"/>
@@ -4457,7 +4457,7 @@
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="LineChartTable" displayName="LineChartTable" ref="A1:C5" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:C13"/>
+  <autoFilter ref="A1:C5"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Date" dataDxfId="1"/>
     <tableColumn id="2" name="2024"/>
@@ -4469,7 +4469,7 @@
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PieChartTable" displayName="PieChartTable" ref="A1:B5" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:B7"/>
+  <autoFilter ref="A1:B5"/>
   <tableColumns count="2">
     <tableColumn id="1" name="Company"/>
     <tableColumn id="2" name="Market Share"/>
@@ -4480,7 +4480,7 @@
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="BarChartTable" displayName="BarChartTable" ref="A1:B4" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:B9"/>
+  <autoFilter ref="A1:B4"/>
   <tableColumns count="2">
     <tableColumn id="1" name="Department"/>
     <tableColumn id="2" name="Employees"/>
@@ -4491,7 +4491,7 @@
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="AreaChartTable" displayName="AreaChartTable" ref="A1:D5" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:D9"/>
+  <autoFilter ref="A1:D5"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Week"/>
     <tableColumn id="2" name="Desktop"/>
@@ -4504,7 +4504,7 @@
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ScatterChartTable" displayName="ScatterChartTable" ref="A1:C5" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:C11"/>
+  <autoFilter ref="A1:C5"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Product"/>
     <tableColumn id="2" name="Price ($)"/>
@@ -4516,7 +4516,7 @@
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="DoughnutChartTable" displayName="DoughnutChartTable" ref="A1:B5" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:B7"/>
+  <autoFilter ref="A1:B5"/>
   <tableColumns count="2">
     <tableColumn id="1" name="Category"/>
     <tableColumn id="2" name="Budget"/>
@@ -4527,7 +4527,7 @@
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="StackedColumnChartTable" displayName="StackedColumnChartTable" ref="A1:E3" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:E5"/>
+  <autoFilter ref="A1:E3"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Quarter"/>
     <tableColumn id="2" name="Electronics"/>
@@ -4541,7 +4541,7 @@
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="ComboChartTable" displayName="ComboChartTable" ref="A1:C4" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:C13"/>
+  <autoFilter ref="A1:C4"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Date" dataDxfId="0"/>
     <tableColumn id="2" name="Revenue"/>

</xml_diff>